<commit_message>
Add uc_ma to the 2026Q2 vintage
uc_ma, estimated at 0750115 on the inputs archived with 2026Q2, joins the
vintage's trend inflation files, workbook, diagnostics, guardrail report
and figures. Every value 2026Q2 had already published is unchanged,
checked row by row against the committed files: the other five models'
series, diagnostics and metadata entries are identical, and the one
guardrail row that changes counts six distinct seeds.

metadata.json keeps the release's own stamp and records the amendment.
Tag v2026Q2 keeps the original five-model files.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/estimates/current/trend_cycle_estimates.xlsx
+++ b/estimates/current/trend_cycle_estimates.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="13" uniqueCount="10">
   <si>
     <t>trend inflation, posterior mean, vintage 2026Q2</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t>biuc_lrexp</t>
+  </si>
+  <si>
+    <t>uc_ma</t>
   </si>
   <si>
     <t>output gap, posterior mean, vintage 2026Q2</t>
@@ -87,7 +90,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D319"/>
+  <dimension ref="A1:E319"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="true"/>
@@ -429,6 +432,9 @@
       <c r="D2" s="0" t="s">
         <v>4</v>
       </c>
+      <c r="E2" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
@@ -439,6 +445,9 @@
       </c>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
+      <c r="E3" s="0">
+        <v>2.0272524920073218</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
@@ -451,6 +460,9 @@
         <v>1.7861553365228513</v>
       </c>
       <c r="D4" s="0"/>
+      <c r="E4" s="0">
+        <v>2.0441700798592621</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
@@ -463,6 +475,9 @@
         <v>1.7930468387452689</v>
       </c>
       <c r="D5" s="0"/>
+      <c r="E5" s="0">
+        <v>2.0409945938977301</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
@@ -475,6 +490,9 @@
         <v>1.7859870680729098</v>
       </c>
       <c r="D6" s="0"/>
+      <c r="E6" s="0">
+        <v>2.0170812745532456</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
@@ -487,6 +505,9 @@
         <v>1.775724675432383</v>
       </c>
       <c r="D7" s="0"/>
+      <c r="E7" s="0">
+        <v>1.9945811318401476</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
@@ -499,6 +520,9 @@
         <v>1.7753816188069653</v>
       </c>
       <c r="D8" s="0"/>
+      <c r="E8" s="0">
+        <v>1.9699508949185456</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
@@ -511,6 +535,9 @@
         <v>1.760124563571799</v>
       </c>
       <c r="D9" s="0"/>
+      <c r="E9" s="0">
+        <v>1.9029814997653458</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
@@ -523,6 +550,9 @@
         <v>1.7582310762328677</v>
       </c>
       <c r="D10" s="0"/>
+      <c r="E10" s="0">
+        <v>1.8507175277682058</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
@@ -535,6 +565,9 @@
         <v>1.7548288824923066</v>
       </c>
       <c r="D11" s="0"/>
+      <c r="E11" s="0">
+        <v>1.8362892332036922</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
@@ -547,6 +580,9 @@
         <v>1.7564589290345265</v>
       </c>
       <c r="D12" s="0"/>
+      <c r="E12" s="0">
+        <v>1.8372409006853692</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
@@ -559,6 +595,9 @@
         <v>1.7624241382299084</v>
       </c>
       <c r="D13" s="0"/>
+      <c r="E13" s="0">
+        <v>1.8467181720380495</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
@@ -571,6 +610,9 @@
         <v>1.7670942014978361</v>
       </c>
       <c r="D14" s="0"/>
+      <c r="E14" s="0">
+        <v>1.8641372450486522</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
@@ -583,6 +625,9 @@
         <v>1.7716799118879802</v>
       </c>
       <c r="D15" s="0"/>
+      <c r="E15" s="0">
+        <v>1.879220566333806</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
@@ -595,6 +640,9 @@
         <v>1.7829956247050649</v>
       </c>
       <c r="D16" s="0"/>
+      <c r="E16" s="0">
+        <v>1.9204442478325832</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1">
@@ -607,6 +655,9 @@
         <v>1.7816120750670204</v>
       </c>
       <c r="D17" s="0"/>
+      <c r="E17" s="0">
+        <v>1.9290721608485726</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1">
@@ -619,6 +670,9 @@
         <v>1.7844517087518883</v>
       </c>
       <c r="D18" s="0"/>
+      <c r="E18" s="0">
+        <v>1.9328658182885912</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1">
@@ -631,6 +685,9 @@
         <v>1.7678554487279283</v>
       </c>
       <c r="D19" s="0"/>
+      <c r="E19" s="0">
+        <v>1.8882928160244024</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1">
@@ -643,6 +700,9 @@
         <v>1.7584499746051774</v>
       </c>
       <c r="D20" s="0"/>
+      <c r="E20" s="0">
+        <v>1.8396306791648105</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1">
@@ -655,6 +715,9 @@
         <v>1.7603716762382629</v>
       </c>
       <c r="D21" s="0"/>
+      <c r="E21" s="0">
+        <v>1.8096802831732495</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1">
@@ -667,6 +730,9 @@
         <v>1.7433760180441487</v>
       </c>
       <c r="D22" s="0"/>
+      <c r="E22" s="0">
+        <v>1.743357765841032</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1">
@@ -679,6 +745,9 @@
         <v>1.7308772912508181</v>
       </c>
       <c r="D23" s="0"/>
+      <c r="E23" s="0">
+        <v>1.6782508835598973</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1">
@@ -691,6 +760,9 @@
         <v>1.7308447544367966</v>
       </c>
       <c r="D24" s="0"/>
+      <c r="E24" s="0">
+        <v>1.6466639760173114</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1">
@@ -703,6 +775,9 @@
         <v>1.7222664930959384</v>
       </c>
       <c r="D25" s="0"/>
+      <c r="E25" s="0">
+        <v>1.5834019019194889</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1">
@@ -715,6 +790,9 @@
         <v>1.715915075231288</v>
       </c>
       <c r="D26" s="0"/>
+      <c r="E26" s="0">
+        <v>1.5501241196621098</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1">
@@ -727,6 +805,9 @@
         <v>1.7045866384478037</v>
       </c>
       <c r="D27" s="0"/>
+      <c r="E27" s="0">
+        <v>1.4936940833800745</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1">
@@ -739,6 +820,9 @@
         <v>1.7052218610853309</v>
       </c>
       <c r="D28" s="0"/>
+      <c r="E28" s="0">
+        <v>1.4706682292565205</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1">
@@ -751,6 +835,9 @@
         <v>1.7020468686095589</v>
       </c>
       <c r="D29" s="0"/>
+      <c r="E29" s="0">
+        <v>1.412810412199611</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1">
@@ -763,6 +850,9 @@
         <v>1.7004165049458018</v>
       </c>
       <c r="D30" s="0"/>
+      <c r="E30" s="0">
+        <v>1.3886678487928448</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1">
@@ -775,6 +865,9 @@
         <v>1.6800746286572503</v>
       </c>
       <c r="D31" s="0"/>
+      <c r="E31" s="0">
+        <v>1.312741761006492</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1">
@@ -787,6 +880,9 @@
         <v>1.677387171766598</v>
       </c>
       <c r="D32" s="0"/>
+      <c r="E32" s="0">
+        <v>1.2856758544220992</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1">
@@ -799,6 +895,9 @@
         <v>1.6887375809265293</v>
       </c>
       <c r="D33" s="0"/>
+      <c r="E33" s="0">
+        <v>1.312094739264726</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1">
@@ -811,6 +910,9 @@
         <v>1.7114087365392452</v>
       </c>
       <c r="D34" s="0"/>
+      <c r="E34" s="0">
+        <v>1.3911124059897584</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1">
@@ -823,6 +925,9 @@
         <v>1.7145907662008639</v>
       </c>
       <c r="D35" s="0"/>
+      <c r="E35" s="0">
+        <v>1.4353875106711205</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1">
@@ -835,6 +940,9 @@
         <v>1.7345762096961328</v>
       </c>
       <c r="D36" s="0"/>
+      <c r="E36" s="0">
+        <v>1.5334968739342214</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1">
@@ -847,6 +955,9 @@
         <v>1.7483775582866559</v>
       </c>
       <c r="D37" s="0"/>
+      <c r="E37" s="0">
+        <v>1.6053808512534962</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1">
@@ -859,6 +970,9 @@
         <v>1.7713360543792833</v>
       </c>
       <c r="D38" s="0"/>
+      <c r="E38" s="0">
+        <v>1.716447094881824</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1">
@@ -871,6 +985,9 @@
         <v>1.8008278259353849</v>
       </c>
       <c r="D39" s="0"/>
+      <c r="E39" s="0">
+        <v>1.8364551616940217</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1">
@@ -883,6 +1000,9 @@
         <v>1.8273890177572287</v>
       </c>
       <c r="D40" s="0"/>
+      <c r="E40" s="0">
+        <v>1.9431509799104578</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1">
@@ -895,6 +1015,9 @@
         <v>1.8212318208380114</v>
       </c>
       <c r="D41" s="0"/>
+      <c r="E41" s="0">
+        <v>1.9556237085910544</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1">
@@ -907,6 +1030,9 @@
         <v>1.8427581407086102</v>
       </c>
       <c r="D42" s="0"/>
+      <c r="E42" s="0">
+        <v>2.0081577976914815</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1">
@@ -919,6 +1045,9 @@
         <v>1.832338537217705</v>
       </c>
       <c r="D43" s="0"/>
+      <c r="E43" s="0">
+        <v>1.9867928778817787</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1">
@@ -931,6 +1060,9 @@
         <v>1.8321313233406056</v>
       </c>
       <c r="D44" s="0"/>
+      <c r="E44" s="0">
+        <v>1.9921394332746085</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1">
@@ -943,6 +1075,9 @@
         <v>1.8233037167470429</v>
       </c>
       <c r="D45" s="0"/>
+      <c r="E45" s="0">
+        <v>1.9454252945318049</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1">
@@ -955,6 +1090,9 @@
         <v>1.8304282295494243</v>
       </c>
       <c r="D46" s="0"/>
+      <c r="E46" s="0">
+        <v>1.9384883894675089</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1">
@@ -967,6 +1105,9 @@
         <v>1.7892793573968613</v>
       </c>
       <c r="D47" s="0"/>
+      <c r="E47" s="0">
+        <v>1.8152148990718624</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1">
@@ -979,6 +1120,9 @@
         <v>1.7717812556144588</v>
       </c>
       <c r="D48" s="0"/>
+      <c r="E48" s="0">
+        <v>1.7492615162329963</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1">
@@ -991,6 +1135,9 @@
         <v>1.7599428407809417</v>
       </c>
       <c r="D49" s="0"/>
+      <c r="E49" s="0">
+        <v>1.6886162640758873</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1">
@@ -1003,6 +1150,9 @@
         <v>1.7778699194911924</v>
       </c>
       <c r="D50" s="0"/>
+      <c r="E50" s="0">
+        <v>1.7272008825749103</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1">
@@ -1015,6 +1165,9 @@
         <v>1.7600889811929856</v>
       </c>
       <c r="D51" s="0"/>
+      <c r="E51" s="0">
+        <v>1.6642749959653393</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1">
@@ -1027,6 +1180,9 @@
         <v>1.7613698979276575</v>
       </c>
       <c r="D52" s="0"/>
+      <c r="E52" s="0">
+        <v>1.6539133555367247</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1">
@@ -1039,6 +1195,9 @@
         <v>1.7483874716960697</v>
       </c>
       <c r="D53" s="0"/>
+      <c r="E53" s="0">
+        <v>1.5926590865106876</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1">
@@ -1051,6 +1210,9 @@
         <v>1.7169072872828417</v>
       </c>
       <c r="D54" s="0"/>
+      <c r="E54" s="0">
+        <v>1.4848465842449905</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1">
@@ -1065,6 +1227,9 @@
       <c r="D55" s="0">
         <v>1.4240029928657123</v>
       </c>
+      <c r="E55" s="0">
+        <v>1.5093723144713973</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1">
@@ -1079,6 +1244,9 @@
       <c r="D56" s="0">
         <v>1.427250016009529</v>
       </c>
+      <c r="E56" s="0">
+        <v>1.4205284957324802</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1">
@@ -1093,6 +1261,9 @@
       <c r="D57" s="0">
         <v>1.4334536664233486</v>
       </c>
+      <c r="E57" s="0">
+        <v>1.3705856069724618</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1">
@@ -1107,6 +1278,9 @@
       <c r="D58" s="0">
         <v>1.4332178815037446</v>
       </c>
+      <c r="E58" s="0">
+        <v>1.2648594296640359</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1">
@@ -1121,6 +1295,9 @@
       <c r="D59" s="0">
         <v>1.433235052237924</v>
       </c>
+      <c r="E59" s="0">
+        <v>1.1832893968270017</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1">
@@ -1135,6 +1312,9 @@
       <c r="D60" s="0">
         <v>1.4433435157769958</v>
       </c>
+      <c r="E60" s="0">
+        <v>1.2528777217255704</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1">
@@ -1149,6 +1329,9 @@
       <c r="D61" s="0">
         <v>1.4434090857632902</v>
       </c>
+      <c r="E61" s="0">
+        <v>1.1865636561804449</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1">
@@ -1163,6 +1346,9 @@
       <c r="D62" s="0">
         <v>1.4534183262318199</v>
       </c>
+      <c r="E62" s="0">
+        <v>1.2903076483757414</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1">
@@ -1177,6 +1363,9 @@
       <c r="D63" s="0">
         <v>1.4565291587634615</v>
       </c>
+      <c r="E63" s="0">
+        <v>1.2807140587367554</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1">
@@ -1191,6 +1380,9 @@
       <c r="D64" s="0">
         <v>1.4593417399318023</v>
       </c>
+      <c r="E64" s="0">
+        <v>1.2880966788206154</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1">
@@ -1205,6 +1397,9 @@
       <c r="D65" s="0">
         <v>1.4646764294142301</v>
       </c>
+      <c r="E65" s="0">
+        <v>1.2957582714481135</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1">
@@ -1219,6 +1414,9 @@
       <c r="D66" s="0">
         <v>1.4686274216258126</v>
       </c>
+      <c r="E66" s="0">
+        <v>1.3234533823558103</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1">
@@ -1233,6 +1431,9 @@
       <c r="D67" s="0">
         <v>1.4709768522244868</v>
       </c>
+      <c r="E67" s="0">
+        <v>1.3020226248072226</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1">
@@ -1247,6 +1448,9 @@
       <c r="D68" s="0">
         <v>1.4816477474478167</v>
       </c>
+      <c r="E68" s="0">
+        <v>1.453943455054973</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1">
@@ -1261,6 +1465,9 @@
       <c r="D69" s="0">
         <v>1.4846160165153564</v>
       </c>
+      <c r="E69" s="0">
+        <v>1.4478803307968817</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1">
@@ -1275,6 +1482,9 @@
       <c r="D70" s="0">
         <v>1.4914407709733357</v>
       </c>
+      <c r="E70" s="0">
+        <v>1.5278139404275153</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1">
@@ -1289,6 +1499,9 @@
       <c r="D71" s="0">
         <v>1.4916589906928266</v>
       </c>
+      <c r="E71" s="0">
+        <v>1.4530304751916954</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1">
@@ -1303,6 +1516,9 @@
       <c r="D72" s="0">
         <v>1.4989831391868467</v>
       </c>
+      <c r="E72" s="0">
+        <v>1.5431245027260048</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1">
@@ -1317,6 +1533,9 @@
       <c r="D73" s="0">
         <v>1.5039576542900099</v>
       </c>
+      <c r="E73" s="0">
+        <v>1.6029258098743542</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1">
@@ -1331,6 +1550,9 @@
       <c r="D74" s="0">
         <v>1.5094265000356353</v>
       </c>
+      <c r="E74" s="0">
+        <v>1.69114724185475</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1">
@@ -1345,6 +1567,9 @@
       <c r="D75" s="0">
         <v>1.5185417404007988</v>
       </c>
+      <c r="E75" s="0">
+        <v>1.8462905041539899</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1">
@@ -1359,6 +1584,9 @@
       <c r="D76" s="0">
         <v>1.5210902149169976</v>
       </c>
+      <c r="E76" s="0">
+        <v>1.9437803941563683</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1">
@@ -1373,6 +1601,9 @@
       <c r="D77" s="0">
         <v>1.5252086489770387</v>
       </c>
+      <c r="E77" s="0">
+        <v>2.0836178015839089</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1">
@@ -1387,6 +1618,9 @@
       <c r="D78" s="0">
         <v>1.5401394361029324</v>
       </c>
+      <c r="E78" s="0">
+        <v>2.3918761762332519</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1">
@@ -1401,6 +1635,9 @@
       <c r="D79" s="0">
         <v>1.5453278085347255</v>
       </c>
+      <c r="E79" s="0">
+        <v>2.5503752381416227</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1">
@@ -1415,6 +1652,9 @@
       <c r="D80" s="0">
         <v>1.5499293950742385</v>
       </c>
+      <c r="E80" s="0">
+        <v>2.6636054623761432</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1">
@@ -1429,6 +1669,9 @@
       <c r="D81" s="0">
         <v>1.5560447583644559</v>
       </c>
+      <c r="E81" s="0">
+        <v>2.7759724578924017</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1">
@@ -1443,6 +1686,9 @@
       <c r="D82" s="0">
         <v>1.5513765648371585</v>
       </c>
+      <c r="E82" s="0">
+        <v>2.7972683897568182</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1">
@@ -1457,6 +1703,9 @@
       <c r="D83" s="0">
         <v>1.5608098204737253</v>
       </c>
+      <c r="E83" s="0">
+        <v>2.9708113698040242</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1">
@@ -1471,6 +1720,9 @@
       <c r="D84" s="0">
         <v>1.5763899821871184</v>
       </c>
+      <c r="E84" s="0">
+        <v>3.2433212960917319</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1">
@@ -1485,6 +1737,9 @@
       <c r="D85" s="0">
         <v>1.5796657694557907</v>
       </c>
+      <c r="E85" s="0">
+        <v>3.4125716977310079</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1">
@@ -1499,6 +1754,9 @@
       <c r="D86" s="0">
         <v>1.6015025403701098</v>
       </c>
+      <c r="E86" s="0">
+        <v>3.6636191191083767</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1">
@@ -1513,6 +1771,9 @@
       <c r="D87" s="0">
         <v>1.6299930732634325</v>
       </c>
+      <c r="E87" s="0">
+        <v>3.7972098045052873</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1">
@@ -1527,6 +1788,9 @@
       <c r="D88" s="0">
         <v>2.2385592368756231</v>
       </c>
+      <c r="E88" s="0">
+        <v>3.9430819382373499</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1">
@@ -1541,6 +1805,9 @@
       <c r="D89" s="0">
         <v>2.2781050619774299</v>
       </c>
+      <c r="E89" s="0">
+        <v>4.0777493694135654</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1">
@@ -1555,6 +1822,9 @@
       <c r="D90" s="0">
         <v>2.3021102327454361</v>
       </c>
+      <c r="E90" s="0">
+        <v>4.1447939013937329</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1">
@@ -1569,6 +1839,9 @@
       <c r="D91" s="0">
         <v>2.39672529550473</v>
       </c>
+      <c r="E91" s="0">
+        <v>4.3298831779957858</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1">
@@ -1583,6 +1856,9 @@
       <c r="D92" s="0">
         <v>2.4495493093153855</v>
       </c>
+      <c r="E92" s="0">
+        <v>4.3828010249626708</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1">
@@ -1597,6 +1873,9 @@
       <c r="D93" s="0">
         <v>2.4619288156109338</v>
       </c>
+      <c r="E93" s="0">
+        <v>4.4000035855247894</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1">
@@ -1611,6 +1890,9 @@
       <c r="D94" s="0">
         <v>2.4762534563752046</v>
       </c>
+      <c r="E94" s="0">
+        <v>4.4166090393582529</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1">
@@ -1625,6 +1907,9 @@
       <c r="D95" s="0">
         <v>2.4930710631666813</v>
       </c>
+      <c r="E95" s="0">
+        <v>4.4259910655608898</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1">
@@ -1639,6 +1924,9 @@
       <c r="D96" s="0">
         <v>2.6138520640112035</v>
       </c>
+      <c r="E96" s="0">
+        <v>4.3983015234049043</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1">
@@ -1653,6 +1941,9 @@
       <c r="D97" s="0">
         <v>2.815585404973167</v>
       </c>
+      <c r="E97" s="0">
+        <v>4.4781300975437155</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1">
@@ -1667,6 +1958,9 @@
       <c r="D98" s="0">
         <v>2.8273102233531877</v>
       </c>
+      <c r="E98" s="0">
+        <v>4.4420898615592188</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1">
@@ -1681,6 +1975,9 @@
       <c r="D99" s="0">
         <v>2.8495723117763312</v>
       </c>
+      <c r="E99" s="0">
+        <v>4.5021532830284103</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1">
@@ -1695,6 +1992,9 @@
       <c r="D100" s="0">
         <v>2.8649561292123047</v>
       </c>
+      <c r="E100" s="0">
+        <v>4.5179161763154188</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1">
@@ -1709,6 +2009,9 @@
       <c r="D101" s="0">
         <v>3.1424416405143849</v>
       </c>
+      <c r="E101" s="0">
+        <v>4.5436633341167418</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1">
@@ -1723,6 +2026,9 @@
       <c r="D102" s="0">
         <v>3.1694455014408764</v>
       </c>
+      <c r="E102" s="0">
+        <v>4.6585930362192825</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1">
@@ -1737,6 +2043,9 @@
       <c r="D103" s="0">
         <v>3.1806988770591915</v>
       </c>
+      <c r="E103" s="0">
+        <v>4.7415680690165907</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1">
@@ -1751,6 +2060,9 @@
       <c r="D104" s="0">
         <v>3.2040476054414855</v>
       </c>
+      <c r="E104" s="0">
+        <v>4.9031844355298349</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1">
@@ -1765,6 +2077,9 @@
       <c r="D105" s="0">
         <v>3.5078450775513206</v>
       </c>
+      <c r="E105" s="0">
+        <v>5.0701245484383755</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1">
@@ -1779,6 +2094,9 @@
       <c r="D106" s="0">
         <v>3.5323148610813044</v>
       </c>
+      <c r="E106" s="0">
+        <v>5.2637850001478181</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1">
@@ -1793,6 +2111,9 @@
       <c r="D107" s="0">
         <v>3.5569379788735929</v>
       </c>
+      <c r="E107" s="0">
+        <v>5.4888819660980204</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1">
@@ -1807,6 +2128,9 @@
       <c r="D108" s="0">
         <v>3.5666475262432016</v>
       </c>
+      <c r="E108" s="0">
+        <v>5.672828894820757</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1">
@@ -1821,6 +2145,9 @@
       <c r="D109" s="0">
         <v>3.5881605682881714</v>
       </c>
+      <c r="E109" s="0">
+        <v>5.8354666402414681</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1">
@@ -1835,6 +2162,9 @@
       <c r="D110" s="0">
         <v>3.8302673473872622</v>
       </c>
+      <c r="E110" s="0">
+        <v>5.9854677546012605</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1">
@@ -1849,6 +2179,9 @@
       <c r="D111" s="0">
         <v>4.3204121103073527</v>
       </c>
+      <c r="E111" s="0">
+        <v>6.0742073603299724</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1">
@@ -1863,6 +2196,9 @@
       <c r="D112" s="0">
         <v>4.4677879983024935</v>
       </c>
+      <c r="E112" s="0">
+        <v>6.1542778946425614</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1">
@@ -1877,6 +2213,9 @@
       <c r="D113" s="0">
         <v>4.4881378470924798</v>
       </c>
+      <c r="E113" s="0">
+        <v>6.1882879952986984</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1">
@@ -1891,6 +2230,9 @@
       <c r="D114" s="0">
         <v>4.492937542718173</v>
       </c>
+      <c r="E114" s="0">
+        <v>6.1825010791878059</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1">
@@ -1905,6 +2247,9 @@
       <c r="D115" s="0">
         <v>4.5097506022024252</v>
       </c>
+      <c r="E115" s="0">
+        <v>6.1612421509635578</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1">
@@ -1919,6 +2264,9 @@
       <c r="D116" s="0">
         <v>4.5573358815007374</v>
       </c>
+      <c r="E116" s="0">
+        <v>6.1916436296171522</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1">
@@ -1933,6 +2281,9 @@
       <c r="D117" s="0">
         <v>4.5565818201892121</v>
       </c>
+      <c r="E117" s="0">
+        <v>6.1716757025943023</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1">
@@ -1947,6 +2298,9 @@
       <c r="D118" s="0">
         <v>4.3742930163684681</v>
       </c>
+      <c r="E118" s="0">
+        <v>6.152354359280964</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1">
@@ -1961,6 +2315,9 @@
       <c r="D119" s="0">
         <v>4.0505840903893802</v>
       </c>
+      <c r="E119" s="0">
+        <v>6.1490058775493175</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1">
@@ -1975,6 +2332,9 @@
       <c r="D120" s="0">
         <v>4.1270108045928984</v>
       </c>
+      <c r="E120" s="0">
+        <v>6.2352409227667467</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1">
@@ -1989,6 +2349,9 @@
       <c r="D121" s="0">
         <v>4.1341676987874072</v>
       </c>
+      <c r="E121" s="0">
+        <v>6.2853926132296447</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1">
@@ -2003,6 +2366,9 @@
       <c r="D122" s="0">
         <v>4.1499279509565747</v>
       </c>
+      <c r="E122" s="0">
+        <v>6.3680248779219682</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1">
@@ -2017,6 +2383,9 @@
       <c r="D123" s="0">
         <v>4.2392487687185021</v>
       </c>
+      <c r="E123" s="0">
+        <v>6.4097625034204011</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1">
@@ -2031,6 +2400,9 @@
       <c r="D124" s="0">
         <v>4.4049708702764292</v>
       </c>
+      <c r="E124" s="0">
+        <v>6.4596699930920733</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1">
@@ -2045,6 +2417,9 @@
       <c r="D125" s="0">
         <v>4.4205711282883442</v>
       </c>
+      <c r="E125" s="0">
+        <v>6.5336597392386935</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1">
@@ -2059,6 +2434,9 @@
       <c r="D126" s="0">
         <v>4.5675204936838636</v>
       </c>
+      <c r="E126" s="0">
+        <v>6.6297636973527654</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1">
@@ -2073,6 +2451,9 @@
       <c r="D127" s="0">
         <v>4.840940633545797</v>
       </c>
+      <c r="E127" s="0">
+        <v>6.7236522400316057</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1">
@@ -2087,6 +2468,9 @@
       <c r="D128" s="0">
         <v>4.8534664672881469</v>
       </c>
+      <c r="E128" s="0">
+        <v>6.7674682177385845</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1">
@@ -2101,6 +2485,9 @@
       <c r="D129" s="0">
         <v>5.0339758342831624</v>
       </c>
+      <c r="E129" s="0">
+        <v>6.8489787333274226</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1">
@@ -2115,6 +2502,9 @@
       <c r="D130" s="0">
         <v>5.3696352575290511</v>
       </c>
+      <c r="E130" s="0">
+        <v>6.8852341761333289</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1">
@@ -2129,6 +2519,9 @@
       <c r="D131" s="0">
         <v>5.4029895212919135</v>
       </c>
+      <c r="E131" s="0">
+        <v>6.9551084034225061</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1">
@@ -2143,6 +2536,9 @@
       <c r="D132" s="0">
         <v>5.7723932233337481</v>
       </c>
+      <c r="E132" s="0">
+        <v>6.9590461548292515</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1">
@@ -2157,6 +2553,9 @@
       <c r="D133" s="0">
         <v>5.7803221249719812</v>
       </c>
+      <c r="E133" s="0">
+        <v>6.9267869555802859</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1">
@@ -2171,6 +2570,9 @@
       <c r="D134" s="0">
         <v>5.7962627302371859</v>
       </c>
+      <c r="E134" s="0">
+        <v>6.8834080130608495</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1">
@@ -2185,6 +2587,9 @@
       <c r="D135" s="0">
         <v>5.7853188776637898</v>
       </c>
+      <c r="E135" s="0">
+        <v>6.7777069170552311</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1">
@@ -2199,6 +2604,9 @@
       <c r="D136" s="0">
         <v>5.7857777612448445</v>
       </c>
+      <c r="E136" s="0">
+        <v>6.6777837614183566</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1">
@@ -2213,6 +2621,9 @@
       <c r="D137" s="0">
         <v>6.0013198654492399</v>
       </c>
+      <c r="E137" s="0">
+        <v>6.5391640986008532</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1">
@@ -2227,6 +2638,9 @@
       <c r="D138" s="0">
         <v>6.4144122000667014</v>
       </c>
+      <c r="E138" s="0">
+        <v>6.3944386082490299</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1">
@@ -2241,6 +2655,9 @@
       <c r="D139" s="0">
         <v>6.2362481525296474</v>
       </c>
+      <c r="E139" s="0">
+        <v>6.1659748622469683</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1">
@@ -2255,6 +2672,9 @@
       <c r="D140" s="0">
         <v>6.0698035416323188</v>
       </c>
+      <c r="E140" s="0">
+        <v>5.9641842983392639</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1">
@@ -2269,6 +2689,9 @@
       <c r="D141" s="0">
         <v>6.1123217883532872</v>
       </c>
+      <c r="E141" s="0">
+        <v>5.7297279910391286</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1">
@@ -2283,6 +2706,9 @@
       <c r="D142" s="0">
         <v>5.7309444230174034</v>
       </c>
+      <c r="E142" s="0">
+        <v>5.5101679632870146</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1">
@@ -2297,6 +2723,9 @@
       <c r="D143" s="0">
         <v>5.4498818222570487</v>
       </c>
+      <c r="E143" s="0">
+        <v>5.2945414596180633</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1">
@@ -2311,6 +2740,9 @@
       <c r="D144" s="0">
         <v>5.4408118764996472</v>
       </c>
+      <c r="E144" s="0">
+        <v>5.1303908724664176</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1">
@@ -2325,6 +2757,9 @@
       <c r="D145" s="0">
         <v>5.3065991100604446</v>
       </c>
+      <c r="E145" s="0">
+        <v>4.9015342029298514</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1">
@@ -2339,6 +2774,9 @@
       <c r="D146" s="0">
         <v>5.1094856153854096</v>
       </c>
+      <c r="E146" s="0">
+        <v>4.7102666995254125</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1">
@@ -2353,6 +2791,9 @@
       <c r="D147" s="0">
         <v>5.2572835132019424</v>
       </c>
+      <c r="E147" s="0">
+        <v>4.556304513443922</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1">
@@ -2367,6 +2808,9 @@
       <c r="D148" s="0">
         <v>5.2816962858305274</v>
       </c>
+      <c r="E148" s="0">
+        <v>4.4485293836081308</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1">
@@ -2381,6 +2825,9 @@
       <c r="D149" s="0">
         <v>5.2650974410174687</v>
       </c>
+      <c r="E149" s="0">
+        <v>4.2514862504060602</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1">
@@ -2395,6 +2842,9 @@
       <c r="D150" s="0">
         <v>5.2088139616741742</v>
       </c>
+      <c r="E150" s="0">
+        <v>4.1600107618148776</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1">
@@ -2409,6 +2859,9 @@
       <c r="D151" s="0">
         <v>5.1322604727452736</v>
       </c>
+      <c r="E151" s="0">
+        <v>4.0081253835538515</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1">
@@ -2423,6 +2876,9 @@
       <c r="D152" s="0">
         <v>4.819558946121683</v>
       </c>
+      <c r="E152" s="0">
+        <v>3.8953796332195148</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1">
@@ -2437,6 +2893,9 @@
       <c r="D153" s="0">
         <v>4.5687907717929352</v>
       </c>
+      <c r="E153" s="0">
+        <v>3.7623767397476704</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1">
@@ -2451,6 +2910,9 @@
       <c r="D154" s="0">
         <v>4.3363200824629926</v>
       </c>
+      <c r="E154" s="0">
+        <v>3.7421779794134551</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1">
@@ -2465,6 +2927,9 @@
       <c r="D155" s="0">
         <v>4.3879104314805479</v>
       </c>
+      <c r="E155" s="0">
+        <v>3.6236863443536467</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1">
@@ -2479,6 +2944,9 @@
       <c r="D156" s="0">
         <v>4.504844900731233</v>
       </c>
+      <c r="E156" s="0">
+        <v>3.5515817430430188</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1">
@@ -2493,6 +2961,9 @@
       <c r="D157" s="0">
         <v>4.4381279086216265</v>
       </c>
+      <c r="E157" s="0">
+        <v>3.4594107504066778</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1">
@@ -2507,6 +2978,9 @@
       <c r="D158" s="0">
         <v>4.2198776643251508</v>
       </c>
+      <c r="E158" s="0">
+        <v>3.3987277917367775</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1">
@@ -2521,6 +2995,9 @@
       <c r="D159" s="0">
         <v>4.1738047477544438</v>
       </c>
+      <c r="E159" s="0">
+        <v>3.2972208309217814</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1">
@@ -2535,6 +3012,9 @@
       <c r="D160" s="0">
         <v>4.0908143080445827</v>
       </c>
+      <c r="E160" s="0">
+        <v>3.3529280041657361</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1">
@@ -2549,6 +3029,9 @@
       <c r="D161" s="0">
         <v>4.0738471693900698</v>
       </c>
+      <c r="E161" s="0">
+        <v>3.3790153769088067</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1">
@@ -2563,6 +3046,9 @@
       <c r="D162" s="0">
         <v>4.1756771902366579</v>
       </c>
+      <c r="E162" s="0">
+        <v>3.4868159498656191</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1">
@@ -2577,6 +3063,9 @@
       <c r="D163" s="0">
         <v>4.1755761499005892</v>
       </c>
+      <c r="E163" s="0">
+        <v>3.5360378690220551</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1">
@@ -2591,6 +3080,9 @@
       <c r="D164" s="0">
         <v>4.2676224140298711</v>
       </c>
+      <c r="E164" s="0">
+        <v>3.5887467608431831</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1">
@@ -2605,6 +3097,9 @@
       <c r="D165" s="0">
         <v>4.0624905025958773</v>
       </c>
+      <c r="E165" s="0">
+        <v>3.6192430727737839</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1">
@@ -2619,6 +3114,9 @@
       <c r="D166" s="0">
         <v>4.0963123311675673</v>
       </c>
+      <c r="E166" s="0">
+        <v>3.6429458440514244</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1">
@@ -2633,6 +3131,9 @@
       <c r="D167" s="0">
         <v>3.9767559790900826</v>
       </c>
+      <c r="E167" s="0">
+        <v>3.7417813347050255</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1">
@@ -2647,6 +3148,9 @@
       <c r="D168" s="0">
         <v>3.8886143888958169</v>
       </c>
+      <c r="E168" s="0">
+        <v>3.8021298736090392</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1">
@@ -2661,6 +3165,9 @@
       <c r="D169" s="0">
         <v>3.7223161600898473</v>
       </c>
+      <c r="E169" s="0">
+        <v>3.7874976885891827</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1">
@@ -2675,6 +3182,9 @@
       <c r="D170" s="0">
         <v>3.7176317942245394</v>
       </c>
+      <c r="E170" s="0">
+        <v>3.794932471700343</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1">
@@ -2689,6 +3199,9 @@
       <c r="D171" s="0">
         <v>3.725673819016468</v>
       </c>
+      <c r="E171" s="0">
+        <v>3.7808992508713062</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1">
@@ -2703,6 +3216,9 @@
       <c r="D172" s="0">
         <v>3.5718588170891001</v>
       </c>
+      <c r="E172" s="0">
+        <v>3.6791757759316171</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1">
@@ -2717,6 +3233,9 @@
       <c r="D173" s="0">
         <v>3.422446460038981</v>
       </c>
+      <c r="E173" s="0">
+        <v>3.6332419071211977</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1">
@@ -2731,6 +3250,9 @@
       <c r="D174" s="0">
         <v>3.2692516529860525</v>
       </c>
+      <c r="E174" s="0">
+        <v>3.644523371368825</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1">
@@ -2745,6 +3267,9 @@
       <c r="D175" s="0">
         <v>3.3632696731313563</v>
       </c>
+      <c r="E175" s="0">
+        <v>3.5339624803721121</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1">
@@ -2759,6 +3284,9 @@
       <c r="D176" s="0">
         <v>3.4175426160643205</v>
       </c>
+      <c r="E176" s="0">
+        <v>3.4734036027526392</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1">
@@ -2773,6 +3301,9 @@
       <c r="D177" s="0">
         <v>3.3541559671985595</v>
       </c>
+      <c r="E177" s="0">
+        <v>3.3530759846042302</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1">
@@ -2787,6 +3318,9 @@
       <c r="D178" s="0">
         <v>3.3259523880095898</v>
       </c>
+      <c r="E178" s="0">
+        <v>3.1237136364406335</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1">
@@ -2801,6 +3335,9 @@
       <c r="D179" s="0">
         <v>3.3125240793072295</v>
       </c>
+      <c r="E179" s="0">
+        <v>3.0175976086807705</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1">
@@ -2815,6 +3352,9 @@
       <c r="D180" s="0">
         <v>3.144757245543814</v>
       </c>
+      <c r="E180" s="0">
+        <v>2.9208433726481911</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1">
@@ -2829,6 +3369,9 @@
       <c r="D181" s="0">
         <v>3.0715380986355063</v>
       </c>
+      <c r="E181" s="0">
+        <v>2.8427262508079667</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1">
@@ -2843,6 +3386,9 @@
       <c r="D182" s="0">
         <v>2.879401040632978</v>
       </c>
+      <c r="E182" s="0">
+        <v>2.7471674572213387</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1">
@@ -2857,6 +3403,9 @@
       <c r="D183" s="0">
         <v>2.9594304360958779</v>
       </c>
+      <c r="E183" s="0">
+        <v>2.6916495929597262</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1">
@@ -2871,6 +3420,9 @@
       <c r="D184" s="0">
         <v>2.854637550911606</v>
       </c>
+      <c r="E184" s="0">
+        <v>2.5964736802431418</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1">
@@ -2885,6 +3437,9 @@
       <c r="D185" s="0">
         <v>2.7566300787156743</v>
       </c>
+      <c r="E185" s="0">
+        <v>2.569452856741008</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1">
@@ -2899,6 +3454,9 @@
       <c r="D186" s="0">
         <v>2.6800775176015197</v>
       </c>
+      <c r="E186" s="0">
+        <v>2.4395946624285183</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1">
@@ -2913,6 +3471,9 @@
       <c r="D187" s="0">
         <v>2.7596917118453654</v>
       </c>
+      <c r="E187" s="0">
+        <v>2.4202387133105305</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1">
@@ -2927,6 +3488,9 @@
       <c r="D188" s="0">
         <v>2.611965787370198</v>
       </c>
+      <c r="E188" s="0">
+        <v>2.2408464650661153</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1">
@@ -2941,6 +3505,9 @@
       <c r="D189" s="0">
         <v>2.5984234536564244</v>
       </c>
+      <c r="E189" s="0">
+        <v>2.2473266194011496</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1">
@@ -2955,6 +3522,9 @@
       <c r="D190" s="0">
         <v>2.5782978910216601</v>
       </c>
+      <c r="E190" s="0">
+        <v>2.1196797186444001</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1">
@@ -2969,6 +3539,9 @@
       <c r="D191" s="0">
         <v>2.595353158830116</v>
       </c>
+      <c r="E191" s="0">
+        <v>2.1773533408700407</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1">
@@ -2983,6 +3556,9 @@
       <c r="D192" s="0">
         <v>2.585907827104073</v>
       </c>
+      <c r="E192" s="0">
+        <v>2.2209839553604605</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1">
@@ -2997,6 +3573,9 @@
       <c r="D193" s="0">
         <v>2.5633071233497051</v>
       </c>
+      <c r="E193" s="0">
+        <v>2.0915980384398032</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1">
@@ -3011,6 +3590,9 @@
       <c r="D194" s="0">
         <v>2.4564811959610453</v>
       </c>
+      <c r="E194" s="0">
+        <v>2.0785485610048635</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1">
@@ -3025,6 +3607,9 @@
       <c r="D195" s="0">
         <v>2.4568988880211906</v>
       </c>
+      <c r="E195" s="0">
+        <v>2.0874608023059529</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1">
@@ -3039,6 +3624,9 @@
       <c r="D196" s="0">
         <v>2.364597928413076</v>
       </c>
+      <c r="E196" s="0">
+        <v>1.973242655561827</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1">
@@ -3053,6 +3641,9 @@
       <c r="D197" s="0">
         <v>2.2593892549764254</v>
       </c>
+      <c r="E197" s="0">
+        <v>1.9743508542696757</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1">
@@ -3067,6 +3658,9 @@
       <c r="D198" s="0">
         <v>2.2442220959160446</v>
       </c>
+      <c r="E198" s="0">
+        <v>1.9977312055607077</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1">
@@ -3081,6 +3675,9 @@
       <c r="D199" s="0">
         <v>2.2343132649671311</v>
       </c>
+      <c r="E199" s="0">
+        <v>2.0320672920960279</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1">
@@ -3095,6 +3692,9 @@
       <c r="D200" s="0">
         <v>2.2192452794302926</v>
       </c>
+      <c r="E200" s="0">
+        <v>1.8736591847059898</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1">
@@ -3109,6 +3709,9 @@
       <c r="D201" s="0">
         <v>2.2113087885798684</v>
       </c>
+      <c r="E201" s="0">
+        <v>1.8756066631253843</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1">
@@ -3123,6 +3726,9 @@
       <c r="D202" s="0">
         <v>2.1946186934043834</v>
       </c>
+      <c r="E202" s="0">
+        <v>1.6779588219223072</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1">
@@ -3137,6 +3743,9 @@
       <c r="D203" s="0">
         <v>2.1153034656811194</v>
       </c>
+      <c r="E203" s="0">
+        <v>1.5136639243003487</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1">
@@ -3151,6 +3760,9 @@
       <c r="D204" s="0">
         <v>2.1524351827000756</v>
       </c>
+      <c r="E204" s="0">
+        <v>1.3926670452065482</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1">
@@ -3165,6 +3777,9 @@
       <c r="D205" s="0">
         <v>1.9971385907666699</v>
       </c>
+      <c r="E205" s="0">
+        <v>1.3399285337547851</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1">
@@ -3179,6 +3794,9 @@
       <c r="D206" s="0">
         <v>1.9530800106849893</v>
       </c>
+      <c r="E206" s="0">
+        <v>1.2279591013241475</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1">
@@ -3193,6 +3811,9 @@
       <c r="D207" s="0">
         <v>1.9031081690579441</v>
       </c>
+      <c r="E207" s="0">
+        <v>1.2840129192518366</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1">
@@ -3207,6 +3828,9 @@
       <c r="D208" s="0">
         <v>1.8934811991405016</v>
       </c>
+      <c r="E208" s="0">
+        <v>1.3483172383582662</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1">
@@ -3221,6 +3845,9 @@
       <c r="D209" s="0">
         <v>1.8864182377502567</v>
       </c>
+      <c r="E209" s="0">
+        <v>1.4202671827448918</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1">
@@ -3235,6 +3862,9 @@
       <c r="D210" s="0">
         <v>1.820326920661796</v>
       </c>
+      <c r="E210" s="0">
+        <v>1.5103571832727347</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1">
@@ -3249,6 +3879,9 @@
       <c r="D211" s="0">
         <v>1.8876298882154159</v>
       </c>
+      <c r="E211" s="0">
+        <v>1.7467137824575738</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1">
@@ -3263,6 +3896,9 @@
       <c r="D212" s="0">
         <v>1.891307268981135</v>
       </c>
+      <c r="E212" s="0">
+        <v>1.8544116076953818</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1">
@@ -3277,6 +3913,9 @@
       <c r="D213" s="0">
         <v>1.8957914977423296</v>
       </c>
+      <c r="E213" s="0">
+        <v>1.9574460413144665</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1">
@@ -3291,6 +3930,9 @@
       <c r="D214" s="0">
         <v>1.8983639472217995</v>
       </c>
+      <c r="E214" s="0">
+        <v>2.066436651966967</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1">
@@ -3305,6 +3947,9 @@
       <c r="D215" s="0">
         <v>1.8956701879064919</v>
       </c>
+      <c r="E215" s="0">
+        <v>2.0118596415392904</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1">
@@ -3319,6 +3964,9 @@
       <c r="D216" s="0">
         <v>1.8955938413795916</v>
       </c>
+      <c r="E216" s="0">
+        <v>2.0538243373812333</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1">
@@ -3333,6 +3981,9 @@
       <c r="D217" s="0">
         <v>1.894087001991577</v>
       </c>
+      <c r="E217" s="0">
+        <v>1.9978525437081616</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1">
@@ -3347,6 +3998,9 @@
       <c r="D218" s="0">
         <v>1.8943488253013239</v>
       </c>
+      <c r="E218" s="0">
+        <v>1.98409425448808</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1">
@@ -3361,6 +4015,9 @@
       <c r="D219" s="0">
         <v>1.8924530087148455</v>
       </c>
+      <c r="E219" s="0">
+        <v>1.8885686307854834</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1">
@@ -3375,6 +4032,9 @@
       <c r="D220" s="0">
         <v>1.8896470218674237</v>
       </c>
+      <c r="E220" s="0">
+        <v>1.7910714335888269</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1">
@@ -3389,6 +4049,9 @@
       <c r="D221" s="0">
         <v>1.899442789203577</v>
       </c>
+      <c r="E221" s="0">
+        <v>1.7912261526372359</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1">
@@ -3403,6 +4066,9 @@
       <c r="D222" s="0">
         <v>1.890174814395712</v>
       </c>
+      <c r="E222" s="0">
+        <v>1.834480272442103</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1">
@@ -3417,6 +4083,9 @@
       <c r="D223" s="0">
         <v>1.8915036948458344</v>
       </c>
+      <c r="E223" s="0">
+        <v>1.9514876722166219</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1">
@@ -3431,6 +4100,9 @@
       <c r="D224" s="0">
         <v>1.8902184892981948</v>
       </c>
+      <c r="E224" s="0">
+        <v>1.9909156264830994</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1">
@@ -3445,6 +4117,9 @@
       <c r="D225" s="0">
         <v>1.8810488594833184</v>
       </c>
+      <c r="E225" s="0">
+        <v>2.0316435592502193</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1">
@@ -3459,6 +4134,9 @@
       <c r="D226" s="0">
         <v>1.8919841871041858</v>
       </c>
+      <c r="E226" s="0">
+        <v>2.133726011114641</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1">
@@ -3473,6 +4151,9 @@
       <c r="D227" s="0">
         <v>1.8908125673692606</v>
       </c>
+      <c r="E227" s="0">
+        <v>2.098985839090052</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1">
@@ -3487,6 +4168,9 @@
       <c r="D228" s="0">
         <v>1.8940247589662771</v>
       </c>
+      <c r="E228" s="0">
+        <v>2.2226235202157749</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1">
@@ -3501,6 +4185,9 @@
       <c r="D229" s="0">
         <v>1.8941746703030702</v>
       </c>
+      <c r="E229" s="0">
+        <v>2.2595110373827905</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1">
@@ -3515,6 +4202,9 @@
       <c r="D230" s="0">
         <v>1.8955072197079534</v>
       </c>
+      <c r="E230" s="0">
+        <v>2.359956209312776</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1">
@@ -3529,6 +4219,9 @@
       <c r="D231" s="0">
         <v>1.8953025767003968</v>
       </c>
+      <c r="E231" s="0">
+        <v>2.393418821900807</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1">
@@ -3543,6 +4236,9 @@
       <c r="D232" s="0">
         <v>1.8946714499349873</v>
       </c>
+      <c r="E232" s="0">
+        <v>2.414646217154552</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1">
@@ -3557,6 +4253,9 @@
       <c r="D233" s="0">
         <v>1.8954729608830705</v>
       </c>
+      <c r="E233" s="0">
+        <v>2.4848693726804183</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1">
@@ -3571,6 +4270,9 @@
       <c r="D234" s="0">
         <v>1.8866827764791585</v>
       </c>
+      <c r="E234" s="0">
+        <v>2.4749815613010986</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1">
@@ -3585,6 +4287,9 @@
       <c r="D235" s="0">
         <v>1.8942989570642026</v>
       </c>
+      <c r="E235" s="0">
+        <v>2.5159098290482413</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1">
@@ -3599,6 +4304,9 @@
       <c r="D236" s="0">
         <v>1.8949268963586401</v>
       </c>
+      <c r="E236" s="0">
+        <v>2.5798548293487622</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1">
@@ -3613,6 +4321,9 @@
       <c r="D237" s="0">
         <v>1.8941870704975978</v>
       </c>
+      <c r="E237" s="0">
+        <v>2.5594733760224635</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1">
@@ -3627,6 +4338,9 @@
       <c r="D238" s="0">
         <v>1.8926480123311764</v>
       </c>
+      <c r="E238" s="0">
+        <v>2.5328687558417675</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1">
@@ -3641,6 +4355,9 @@
       <c r="D239" s="0">
         <v>1.8917573392982747</v>
       </c>
+      <c r="E239" s="0">
+        <v>2.5136361958920053</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1">
@@ -3655,6 +4372,9 @@
       <c r="D240" s="0">
         <v>1.8891336249083914</v>
       </c>
+      <c r="E240" s="0">
+        <v>2.4710624229434903</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1">
@@ -3669,6 +4389,9 @@
       <c r="D241" s="0">
         <v>1.8845422972811292</v>
       </c>
+      <c r="E241" s="0">
+        <v>2.3945164032943342</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1">
@@ -3683,6 +4406,9 @@
       <c r="D242" s="0">
         <v>1.8688974725170933</v>
       </c>
+      <c r="E242" s="0">
+        <v>2.4129028423534682</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1">
@@ -3697,6 +4423,9 @@
       <c r="D243" s="0">
         <v>1.8678406141392709</v>
       </c>
+      <c r="E243" s="0">
+        <v>2.3879426270916748</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1">
@@ -3711,6 +4440,9 @@
       <c r="D244" s="0">
         <v>1.8836482853947394</v>
       </c>
+      <c r="E244" s="0">
+        <v>2.3481441512066841</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1">
@@ -3725,6 +4457,9 @@
       <c r="D245" s="0">
         <v>1.8868952022735632</v>
       </c>
+      <c r="E245" s="0">
+        <v>2.3423552193135571</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1">
@@ -3739,6 +4474,9 @@
       <c r="D246" s="0">
         <v>1.9039260865014427</v>
       </c>
+      <c r="E246" s="0">
+        <v>2.2909935933975758</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1">
@@ -3753,6 +4491,9 @@
       <c r="D247" s="0">
         <v>1.9052936889126786</v>
       </c>
+      <c r="E247" s="0">
+        <v>2.242004187704036</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1">
@@ -3767,6 +4508,9 @@
       <c r="D248" s="0">
         <v>1.9047900924034304</v>
       </c>
+      <c r="E248" s="0">
+        <v>2.1895588947457303</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1">
@@ -3781,6 +4525,9 @@
       <c r="D249" s="0">
         <v>1.9017816859848782</v>
       </c>
+      <c r="E249" s="0">
+        <v>2.081169545977378</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1">
@@ -3795,6 +4542,9 @@
       <c r="D250" s="0">
         <v>1.9008543025275366</v>
       </c>
+      <c r="E250" s="0">
+        <v>2.0502309465597293</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1">
@@ -3809,6 +4559,9 @@
       <c r="D251" s="0">
         <v>1.9090211199053353</v>
       </c>
+      <c r="E251" s="0">
+        <v>2.0421560238828094</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1">
@@ -3823,6 +4576,9 @@
       <c r="D252" s="0">
         <v>1.887833944032866</v>
       </c>
+      <c r="E252" s="0">
+        <v>2.0267795534765454</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1">
@@ -3837,6 +4593,9 @@
       <c r="D253" s="0">
         <v>1.876632689721802</v>
       </c>
+      <c r="E253" s="0">
+        <v>2.0174823227953054</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1">
@@ -3851,6 +4610,9 @@
       <c r="D254" s="0">
         <v>1.8722066182046433</v>
       </c>
+      <c r="E254" s="0">
+        <v>1.9745048968949985</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1">
@@ -3865,6 +4627,9 @@
       <c r="D255" s="0">
         <v>1.8758422575030744</v>
       </c>
+      <c r="E255" s="0">
+        <v>1.9647944564803874</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1">
@@ -3879,6 +4644,9 @@
       <c r="D256" s="0">
         <v>1.8663656982949974</v>
       </c>
+      <c r="E256" s="0">
+        <v>1.9730058912466582</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1">
@@ -3893,6 +4661,9 @@
       <c r="D257" s="0">
         <v>1.8521473916987763</v>
       </c>
+      <c r="E257" s="0">
+        <v>2.016358420476613</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1">
@@ -3907,6 +4678,9 @@
       <c r="D258" s="0">
         <v>1.8691255179237236</v>
       </c>
+      <c r="E258" s="0">
+        <v>2.0250827245069938</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1">
@@ -3921,6 +4695,9 @@
       <c r="D259" s="0">
         <v>1.8970002702948885</v>
       </c>
+      <c r="E259" s="0">
+        <v>2.0134610261569606</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1">
@@ -3935,6 +4712,9 @@
       <c r="D260" s="0">
         <v>1.8934240018392483</v>
       </c>
+      <c r="E260" s="0">
+        <v>1.9118243951086011</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1">
@@ -3949,6 +4729,9 @@
       <c r="D261" s="0">
         <v>1.8761098082492951</v>
       </c>
+      <c r="E261" s="0">
+        <v>1.8289658282183572</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="1">
@@ -3963,6 +4746,9 @@
       <c r="D262" s="0">
         <v>1.8732895605581923</v>
       </c>
+      <c r="E262" s="0">
+        <v>1.795934202742858</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="1">
@@ -3977,6 +4763,9 @@
       <c r="D263" s="0">
         <v>1.8757489013202751</v>
       </c>
+      <c r="E263" s="0">
+        <v>1.678445069474509</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1">
@@ -3991,6 +4780,9 @@
       <c r="D264" s="0">
         <v>1.87054819863351</v>
       </c>
+      <c r="E264" s="0">
+        <v>1.6251627391476813</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="1">
@@ -4005,6 +4797,9 @@
       <c r="D265" s="0">
         <v>1.8494299079589178</v>
       </c>
+      <c r="E265" s="0">
+        <v>1.5911020713250841</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="1">
@@ -4019,6 +4814,9 @@
       <c r="D266" s="0">
         <v>1.8267480375668517</v>
       </c>
+      <c r="E266" s="0">
+        <v>1.5101214770729088</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1">
@@ -4033,6 +4831,9 @@
       <c r="D267" s="0">
         <v>1.8202411896337716</v>
       </c>
+      <c r="E267" s="0">
+        <v>1.4155069038419201</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1">
@@ -4047,6 +4848,9 @@
       <c r="D268" s="0">
         <v>1.8177236847553635</v>
       </c>
+      <c r="E268" s="0">
+        <v>1.4330615277082335</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1">
@@ -4061,6 +4865,9 @@
       <c r="D269" s="0">
         <v>1.8155176343920703</v>
       </c>
+      <c r="E269" s="0">
+        <v>1.3914737745356467</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1">
@@ -4075,6 +4882,9 @@
       <c r="D270" s="0">
         <v>1.8142281912959024</v>
       </c>
+      <c r="E270" s="0">
+        <v>1.364782462531466</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1">
@@ -4089,6 +4899,9 @@
       <c r="D271" s="0">
         <v>1.8128890635350945</v>
       </c>
+      <c r="E271" s="0">
+        <v>1.3023904167910876</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1">
@@ -4103,6 +4916,9 @@
       <c r="D272" s="0">
         <v>1.8113791484181061</v>
       </c>
+      <c r="E272" s="0">
+        <v>1.232473053103722</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1">
@@ -4117,6 +4933,9 @@
       <c r="D273" s="0">
         <v>1.8095591150298389</v>
       </c>
+      <c r="E273" s="0">
+        <v>1.1589101687251251</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="1">
@@ -4131,6 +4950,9 @@
       <c r="D274" s="0">
         <v>1.8080326464828553</v>
       </c>
+      <c r="E274" s="0">
+        <v>1.107614540865459</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1">
@@ -4145,6 +4967,9 @@
       <c r="D275" s="0">
         <v>1.8057446958884031</v>
       </c>
+      <c r="E275" s="0">
+        <v>1.1939418014998806</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1">
@@ -4159,6 +4984,9 @@
       <c r="D276" s="0">
         <v>1.8073263916707574</v>
       </c>
+      <c r="E276" s="0">
+        <v>1.198460601471316</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1">
@@ -4173,6 +5001,9 @@
       <c r="D277" s="0">
         <v>1.7914271957617616</v>
       </c>
+      <c r="E277" s="0">
+        <v>1.2323726183203745</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1">
@@ -4187,6 +5018,9 @@
       <c r="D278" s="0">
         <v>1.8043279542038497</v>
       </c>
+      <c r="E278" s="0">
+        <v>1.2959225705104935</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1">
@@ -4201,6 +5035,9 @@
       <c r="D279" s="0">
         <v>1.8136512892124079</v>
       </c>
+      <c r="E279" s="0">
+        <v>1.4290875882007446</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1">
@@ -4215,6 +5052,9 @@
       <c r="D280" s="0">
         <v>1.8172722206146432</v>
       </c>
+      <c r="E280" s="0">
+        <v>1.4807966024486112</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="1">
@@ -4229,6 +5069,9 @@
       <c r="D281" s="0">
         <v>1.82191548851103</v>
       </c>
+      <c r="E281" s="0">
+        <v>1.5633373909619555</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="1">
@@ -4243,6 +5086,9 @@
       <c r="D282" s="0">
         <v>1.8418118765863392</v>
       </c>
+      <c r="E282" s="0">
+        <v>1.6422894321432608</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="1">
@@ -4257,6 +5103,9 @@
       <c r="D283" s="0">
         <v>1.8407698855585759</v>
       </c>
+      <c r="E283" s="0">
+        <v>1.620900540597336</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="1">
@@ -4271,6 +5120,9 @@
       <c r="D284" s="0">
         <v>1.8269170942251338</v>
       </c>
+      <c r="E284" s="0">
+        <v>1.7134644420083462</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="1">
@@ -4285,6 +5137,9 @@
       <c r="D285" s="0">
         <v>1.827340102454865</v>
       </c>
+      <c r="E285" s="0">
+        <v>1.8239533189193891</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="1">
@@ -4299,6 +5154,9 @@
       <c r="D286" s="0">
         <v>1.828202438080953</v>
       </c>
+      <c r="E286" s="0">
+        <v>1.8865636023570818</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="1">
@@ -4313,6 +5171,9 @@
       <c r="D287" s="0">
         <v>1.8292861334574555</v>
       </c>
+      <c r="E287" s="0">
+        <v>1.8905183057731798</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="1">
@@ -4327,6 +5188,9 @@
       <c r="D288" s="0">
         <v>1.8308971329028383</v>
       </c>
+      <c r="E288" s="0">
+        <v>1.8786511519836957</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="1">
@@ -4341,6 +5205,9 @@
       <c r="D289" s="0">
         <v>1.8330030043475276</v>
       </c>
+      <c r="E289" s="0">
+        <v>1.9086418800144207</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="1">
@@ -4355,6 +5222,9 @@
       <c r="D290" s="0">
         <v>1.8348659729363466</v>
       </c>
+      <c r="E290" s="0">
+        <v>1.9198282838894769</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="1">
@@ -4369,6 +5239,9 @@
       <c r="D291" s="0">
         <v>1.837932373740222</v>
       </c>
+      <c r="E291" s="0">
+        <v>2.0167207780827878</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="1">
@@ -4383,6 +5256,9 @@
       <c r="D292" s="0">
         <v>1.8396974893482971</v>
       </c>
+      <c r="E292" s="0">
+        <v>2.0597471068518578</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="1">
@@ -4397,6 +5273,9 @@
       <c r="D293" s="0">
         <v>1.8409641581578657</v>
       </c>
+      <c r="E293" s="0">
+        <v>2.15615628439964</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="1">
@@ -4411,6 +5290,9 @@
       <c r="D294" s="0">
         <v>1.8405877426782669</v>
       </c>
+      <c r="E294" s="0">
+        <v>2.2706467403977406</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="1">
@@ -4425,6 +5307,9 @@
       <c r="D295" s="0">
         <v>1.8084286384141031</v>
       </c>
+      <c r="E295" s="0">
+        <v>2.3641432142061012</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1">
@@ -4439,6 +5324,9 @@
       <c r="D296" s="0">
         <v>1.8135429165511558</v>
       </c>
+      <c r="E296" s="0">
+        <v>2.5639247003481604</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="1">
@@ -4453,6 +5341,9 @@
       <c r="D297" s="0">
         <v>1.8333892224698691</v>
       </c>
+      <c r="E297" s="0">
+        <v>2.7188533599949132</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="1">
@@ -4467,6 +5358,9 @@
       <c r="D298" s="0">
         <v>1.8805385934098127</v>
       </c>
+      <c r="E298" s="0">
+        <v>2.893263299879822</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1">
@@ -4481,6 +5375,9 @@
       <c r="D299" s="0">
         <v>1.9160937593549752</v>
       </c>
+      <c r="E299" s="0">
+        <v>3.0505125751838742</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1">
@@ -4495,6 +5392,9 @@
       <c r="D300" s="0">
         <v>1.9562888833687948</v>
       </c>
+      <c r="E300" s="0">
+        <v>3.1667333858385613</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1">
@@ -4509,6 +5409,9 @@
       <c r="D301" s="0">
         <v>1.9968126469688683</v>
       </c>
+      <c r="E301" s="0">
+        <v>3.2776260387193434</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="1">
@@ -4523,6 +5426,9 @@
       <c r="D302" s="0">
         <v>1.984068215278991</v>
       </c>
+      <c r="E302" s="0">
+        <v>3.3372738194973652</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="1">
@@ -4537,6 +5443,9 @@
       <c r="D303" s="0">
         <v>2.0507044913130428</v>
       </c>
+      <c r="E303" s="0">
+        <v>3.359556816365648</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="1">
@@ -4551,6 +5460,9 @@
       <c r="D304" s="0">
         <v>2.067456908293368</v>
       </c>
+      <c r="E304" s="0">
+        <v>3.3346427038010877</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="1">
@@ -4565,6 +5477,9 @@
       <c r="D305" s="0">
         <v>2.1038158699334764</v>
       </c>
+      <c r="E305" s="0">
+        <v>3.2845406793345751</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="1">
@@ -4579,6 +5494,9 @@
       <c r="D306" s="0">
         <v>1.9743961161077621</v>
       </c>
+      <c r="E306" s="0">
+        <v>3.2139302023313001</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="1">
@@ -4593,6 +5511,9 @@
       <c r="D307" s="0">
         <v>1.9800099541853953</v>
       </c>
+      <c r="E307" s="0">
+        <v>3.1326984770453401</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="1">
@@ -4607,6 +5528,9 @@
       <c r="D308" s="0">
         <v>1.9721822744283899</v>
       </c>
+      <c r="E308" s="0">
+        <v>3.0877594046751189</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="1">
@@ -4621,6 +5545,9 @@
       <c r="D309" s="0">
         <v>1.9730964225786867</v>
       </c>
+      <c r="E309" s="0">
+        <v>3.0239688008760748</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="1">
@@ -4635,6 +5562,9 @@
       <c r="D310" s="0">
         <v>1.9134719214862748</v>
       </c>
+      <c r="E310" s="0">
+        <v>3.0426038409335261</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="1">
@@ -4649,6 +5579,9 @@
       <c r="D311" s="0">
         <v>1.9367837745143957</v>
       </c>
+      <c r="E311" s="0">
+        <v>2.985555065276142</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="1">
@@ -4663,6 +5596,9 @@
       <c r="D312" s="0">
         <v>1.9361952126037738</v>
       </c>
+      <c r="E312" s="0">
+        <v>2.9682829405105631</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="1">
@@ -4677,6 +5613,9 @@
       <c r="D313" s="0">
         <v>1.9417993711102648</v>
       </c>
+      <c r="E313" s="0">
+        <v>3.0069340142176859</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="1">
@@ -4691,6 +5630,9 @@
       <c r="D314" s="0">
         <v>1.9500637828082954</v>
       </c>
+      <c r="E314" s="0">
+        <v>3.0853074561828771</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="1">
@@ -4705,6 +5647,9 @@
       <c r="D315" s="0">
         <v>1.975695112619644</v>
       </c>
+      <c r="E315" s="0">
+        <v>3.0768726910488513</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="1">
@@ -4719,6 +5664,9 @@
       <c r="D316" s="0">
         <v>1.9807841359835976</v>
       </c>
+      <c r="E316" s="0">
+        <v>3.1645762317281276</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="1">
@@ -4733,6 +5681,9 @@
       <c r="D317" s="0">
         <v>1.9834370753968296</v>
       </c>
+      <c r="E317" s="0">
+        <v>3.228974756294476</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="1">
@@ -4747,6 +5698,9 @@
       <c r="D318" s="0">
         <v>1.9869867523545246</v>
       </c>
+      <c r="E318" s="0">
+        <v>3.345035384160493</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="1">
@@ -4759,6 +5713,9 @@
         <v>2.7618741722894713</v>
       </c>
       <c r="D319" s="0"/>
+      <c r="E319" s="0">
+        <v>3.4116639353750387</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -5093,7 +6050,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -5101,10 +6058,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -8937,7 +9894,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
@@ -8945,7 +9902,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">

</xml_diff>